<commit_message>
Add topic 4 GDM
</commit_message>
<xml_diff>
--- a/data/Wilson_Latorre/Data_multi_site_R_course.xlsx
+++ b/data/Wilson_Latorre/Data_multi_site_R_course.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucordoba-my.sharepoint.com/personal/bv2nilud_uco_es/Documents/Docencia/Doctorado-UCO/2025-AEMER-UCO/datos/Wilson_Latorre/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AEMeR-UCO\data\Wilson_Latorre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{5A15BB4B-9CE6-4C74-A494-30313DF406C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E3C8A9C-6BD3-47CF-A363-F913350726EE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4EDEBF7-B056-4260-9B54-070E61C82739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="77">
   <si>
     <t>SU</t>
   </si>
@@ -250,6 +250,12 @@
   </si>
   <si>
     <t>Parcela</t>
+  </si>
+  <si>
+    <t>Long</t>
+  </si>
+  <si>
+    <t>Lat</t>
   </si>
 </sst>
 </file>
@@ -602,14 +608,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -625,8 +631,14 @@
       <c r="E1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -642,8 +654,14 @@
       <c r="E2">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F2">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G2" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -659,8 +677,14 @@
       <c r="E3">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F3">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G3" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -676,8 +700,14 @@
       <c r="E4">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F4">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G4" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -693,8 +723,14 @@
       <c r="E5">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F5">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G5" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -710,8 +746,14 @@
       <c r="E6">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F6">
+        <v>-80.3125</v>
+      </c>
+      <c r="G6" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -727,8 +769,14 @@
       <c r="E7">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F7">
+        <v>-80.3125</v>
+      </c>
+      <c r="G7" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -744,8 +792,14 @@
       <c r="E8">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F8">
+        <v>-80.3125</v>
+      </c>
+      <c r="G8" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -761,8 +815,14 @@
       <c r="E9">
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F9">
+        <v>-80.3125</v>
+      </c>
+      <c r="G9" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -778,8 +838,14 @@
       <c r="E10">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F10">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G10" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -795,8 +861,14 @@
       <c r="E11">
         <v>20</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F11">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G11" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -812,8 +884,14 @@
       <c r="E12">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F12">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G12" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -829,8 +907,14 @@
       <c r="E13">
         <v>20</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F13">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G13" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -846,8 +930,14 @@
       <c r="E14">
         <v>20</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F14">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G14" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -863,8 +953,14 @@
       <c r="E15">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F15">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G15" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -880,8 +976,14 @@
       <c r="E16">
         <v>20</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F16">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G16" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -897,8 +999,14 @@
       <c r="E17">
         <v>20</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F17">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G17" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -914,8 +1022,14 @@
       <c r="E18">
         <v>21</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F18">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G18" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -931,8 +1045,14 @@
       <c r="E19">
         <v>21</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F19">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G19" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -948,8 +1068,14 @@
       <c r="E20">
         <v>21</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F20">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G20" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -965,8 +1091,14 @@
       <c r="E21">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F21">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G21" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -982,8 +1114,14 @@
       <c r="E22">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F22">
+        <v>-80.3125</v>
+      </c>
+      <c r="G22" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -999,8 +1137,14 @@
       <c r="E23">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F23">
+        <v>-80.3125</v>
+      </c>
+      <c r="G23" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1016,8 +1160,14 @@
       <c r="E24">
         <v>21</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F24">
+        <v>-80.3125</v>
+      </c>
+      <c r="G24" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1033,8 +1183,14 @@
       <c r="E25">
         <v>21</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F25">
+        <v>-80.3125</v>
+      </c>
+      <c r="G25" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -1050,8 +1206,14 @@
       <c r="E26">
         <v>21</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F26">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G26" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -1067,8 +1229,14 @@
       <c r="E27">
         <v>21</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F27">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G27" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -1084,8 +1252,14 @@
       <c r="E28">
         <v>21</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F28">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G28" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -1101,8 +1275,14 @@
       <c r="E29">
         <v>21</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F29">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G29" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1118,8 +1298,14 @@
       <c r="E30">
         <v>21</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F30">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G30" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -1135,8 +1321,14 @@
       <c r="E31">
         <v>21</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F31">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G31" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -1152,8 +1344,14 @@
       <c r="E32">
         <v>21</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F32">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G32" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -1169,8 +1367,14 @@
       <c r="E33">
         <v>21</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F33">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G33" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -1186,8 +1390,14 @@
       <c r="E34">
         <v>21</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F34">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G34" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1203,8 +1413,14 @@
       <c r="E35">
         <v>21</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F35">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G35" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1220,8 +1436,14 @@
       <c r="E36">
         <v>21</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F36">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G36" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1237,8 +1459,14 @@
       <c r="E37">
         <v>21</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F37">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G37" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1254,8 +1482,14 @@
       <c r="E38">
         <v>21</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F38">
+        <v>-80.3125</v>
+      </c>
+      <c r="G38" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1271,8 +1505,14 @@
       <c r="E39">
         <v>21</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F39">
+        <v>-80.3125</v>
+      </c>
+      <c r="G39" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1288,8 +1528,14 @@
       <c r="E40">
         <v>21</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F40">
+        <v>-80.3125</v>
+      </c>
+      <c r="G40" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1305,8 +1551,14 @@
       <c r="E41">
         <v>21</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F41">
+        <v>-80.3125</v>
+      </c>
+      <c r="G41" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -1322,8 +1574,14 @@
       <c r="E42">
         <v>21</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F42">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G42" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -1339,8 +1597,14 @@
       <c r="E43">
         <v>21</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F43">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G43" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -1356,8 +1620,14 @@
       <c r="E44">
         <v>21</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F44">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G44" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -1373,8 +1643,14 @@
       <c r="E45">
         <v>21</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F45">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G45" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>50</v>
       </c>
@@ -1390,8 +1666,14 @@
       <c r="E46">
         <v>21</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F46">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G46" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -1407,8 +1689,14 @@
       <c r="E47">
         <v>21</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F47">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G47" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>52</v>
       </c>
@@ -1424,8 +1712,14 @@
       <c r="E48">
         <v>21</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F48">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G48" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>53</v>
       </c>
@@ -1441,8 +1735,14 @@
       <c r="E49">
         <v>21</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F49">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G49" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>54</v>
       </c>
@@ -1458,8 +1758,14 @@
       <c r="E50">
         <v>22</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F50">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G50" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>55</v>
       </c>
@@ -1475,8 +1781,14 @@
       <c r="E51">
         <v>22</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F51">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G51" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>56</v>
       </c>
@@ -1492,8 +1804,14 @@
       <c r="E52">
         <v>22</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F52">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G52" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>57</v>
       </c>
@@ -1509,8 +1827,14 @@
       <c r="E53">
         <v>22</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F53">
+        <v>-80.292500000000004</v>
+      </c>
+      <c r="G53" s="1">
+        <v>-1.2235</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>58</v>
       </c>
@@ -1526,8 +1850,14 @@
       <c r="E54">
         <v>22</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F54">
+        <v>-80.3125</v>
+      </c>
+      <c r="G54" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>59</v>
       </c>
@@ -1543,8 +1873,14 @@
       <c r="E55">
         <v>22</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F55">
+        <v>-80.3125</v>
+      </c>
+      <c r="G55" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>60</v>
       </c>
@@ -1560,8 +1896,14 @@
       <c r="E56">
         <v>22</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F56">
+        <v>-80.3125</v>
+      </c>
+      <c r="G56" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>61</v>
       </c>
@@ -1577,8 +1919,14 @@
       <c r="E57">
         <v>22</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F57">
+        <v>-80.3125</v>
+      </c>
+      <c r="G57" s="1">
+        <v>-1.2915000000000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>62</v>
       </c>
@@ -1594,8 +1942,14 @@
       <c r="E58">
         <v>22</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F58">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G58" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>63</v>
       </c>
@@ -1611,8 +1965,14 @@
       <c r="E59">
         <v>22</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F59">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G59" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>64</v>
       </c>
@@ -1628,8 +1988,14 @@
       <c r="E60">
         <v>22</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F60">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G60" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>65</v>
       </c>
@@ -1645,8 +2011,14 @@
       <c r="E61">
         <v>22</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F61">
+        <v>-80.325999999999993</v>
+      </c>
+      <c r="G61" s="1">
+        <v>-1.2575000000000001</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>66</v>
       </c>
@@ -1662,8 +2034,14 @@
       <c r="E62">
         <v>22</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F62">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G62" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>67</v>
       </c>
@@ -1679,8 +2057,14 @@
       <c r="E63">
         <v>22</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F63">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G63" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>68</v>
       </c>
@@ -1696,8 +2080,14 @@
       <c r="E64">
         <v>22</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F64">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G64" s="1">
+        <v>-1.1725000000000001</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>69</v>
       </c>
@@ -1712,6 +2102,12 @@
       </c>
       <c r="E65">
         <v>22</v>
+      </c>
+      <c r="F65">
+        <v>-80.385499999999993</v>
+      </c>
+      <c r="G65" s="1">
+        <v>-1.1725000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>